<commit_message>
Mark all synthetic data as EXAMPLE
All customer, branch and test email addresses now use the reserved
.example domain (RFC 2606), so no address can belong to a real person.
Every generated letter carries an EXAMPLE watermark and footer.
Data, letters, reports and the slide deck regenerated; results unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RcpasmBE1hvgdead6uZREF
</commit_message>
<xml_diff>
--- a/data/batches/2026-08/send_list.xlsx
+++ b/data/batches/2026-08/send_list.xlsx
@@ -925,454 +925,454 @@
     <t>Utami Wibowo</t>
   </si>
   <si>
-    <t>dimas.nasution608@outlook.com</t>
-  </si>
-  <si>
-    <t>vina.saputra573@gmail.com</t>
-  </si>
-  <si>
-    <t>tika.susanto926@gmail.com</t>
-  </si>
-  <si>
-    <t>nur.lestari650@gmail.com</t>
-  </si>
-  <si>
-    <t>joko.setiawan270@gmail.com</t>
-  </si>
-  <si>
-    <t>joko.nugroho688@gmail.com</t>
-  </si>
-  <si>
-    <t>rahmat.siregar337@gmail.com</t>
-  </si>
-  <si>
-    <t>budi.siregar667@gmail.com</t>
-  </si>
-  <si>
-    <t>yuni.ramadhan958@gmail.com</t>
-  </si>
-  <si>
-    <t>vina.setiawan655@outlook.com</t>
-  </si>
-  <si>
-    <t>budi.simanjuntak706@outlook.com</t>
-  </si>
-  <si>
-    <t>tika.firmansyah424@gmail.com</t>
-  </si>
-  <si>
-    <t>lestari.nugroho532@gmail.com</t>
-  </si>
-  <si>
-    <t>citra.siregar111@outlook.com</t>
-  </si>
-  <si>
-    <t>bayu.utomo296@gmail.com</t>
-  </si>
-  <si>
-    <t>vina.permana689@gmail.com</t>
-  </si>
-  <si>
-    <t>laras.firmansyah350@outlook.com</t>
-  </si>
-  <si>
-    <t>kartika.halim174@outlook.com</t>
-  </si>
-  <si>
-    <t>kartika.nugroho952@gmail.com</t>
-  </si>
-  <si>
-    <t>wahyu.gunawan107@outlook.com</t>
-  </si>
-  <si>
-    <t>irfan.sitompul545@yahoo.co.id</t>
-  </si>
-  <si>
-    <t>fitri.santoso810@outlook.com</t>
-  </si>
-  <si>
-    <t>surya.setiawan771@gmail.com</t>
-  </si>
-  <si>
-    <t>gilang.pratama510@outlook.com</t>
-  </si>
-  <si>
-    <t>surya.daeng364@outlook.com</t>
-  </si>
-  <si>
-    <t>andi.setiawan238.old@gmail.com</t>
-  </si>
-  <si>
-    <t>tika.marpaung805@outlook.com</t>
-  </si>
-  <si>
-    <t>mega.marpaung269@gmail.com</t>
-  </si>
-  <si>
-    <t>hendra.sitompul513@yahoo.co.id</t>
-  </si>
-  <si>
-    <t>mega.firmansyah422@gmail.com</t>
-  </si>
-  <si>
-    <t>rizky.firmansyah364@gmail.com</t>
-  </si>
-  <si>
-    <t>joko.wijaya663@gmail.com</t>
-  </si>
-  <si>
-    <t>fitri.rahayu13@outlook.com</t>
-  </si>
-  <si>
-    <t>yoga.lestari340@yahoo.co.id</t>
-  </si>
-  <si>
-    <t>yuni.saputra879@yahoo.co.id</t>
-  </si>
-  <si>
-    <t>oki.hakim372@outlook.com</t>
-  </si>
-  <si>
-    <t>zaki.nasution210@yahoo.co.id</t>
-  </si>
-  <si>
-    <t>rahmat.siregar757@gmail.com</t>
-  </si>
-  <si>
-    <t>gita.hidayat136@gmail.com</t>
-  </si>
-  <si>
-    <t>laras.ramadhan779@yahoo.co.id</t>
-  </si>
-  <si>
-    <t>tika.wijaya764@gmail.com</t>
-  </si>
-  <si>
-    <t>vina.harahap695@gmail.com</t>
-  </si>
-  <si>
-    <t>lestari.lestari789@gmail.com</t>
-  </si>
-  <si>
-    <t>gilang.daeng87@gmail.com</t>
-  </si>
-  <si>
-    <t>mega.syahputra515@gmail.com</t>
-  </si>
-  <si>
-    <t>irfan.lestari524@gmail.com</t>
-  </si>
-  <si>
-    <t>rina.hakim486@gmail.com</t>
-  </si>
-  <si>
-    <t>utami.saputra534@gmail.com</t>
-  </si>
-  <si>
-    <t>eko.firmansyah611@gmail.com</t>
-  </si>
-  <si>
-    <t>gilang.halim260@gmail.com</t>
-  </si>
-  <si>
-    <t>yuni.daeng514@yahoo.co.id</t>
-  </si>
-  <si>
-    <t>eko.simanjuntak230@outlook.com</t>
-  </si>
-  <si>
-    <t>taufik.purnomo473@gmail.com</t>
-  </si>
-  <si>
-    <t>nur.kusuma124@gmail.com</t>
-  </si>
-  <si>
-    <t>bayu.setiawan607@gmail.com</t>
-  </si>
-  <si>
-    <t>bayu.gunawan728@outlook.com</t>
-  </si>
-  <si>
-    <t>zaki.purnomo501@gmail.com</t>
-  </si>
-  <si>
-    <t>eko.nasution202@gmail.com</t>
-  </si>
-  <si>
-    <t>dewi.hidayat608@gmail.com</t>
-  </si>
-  <si>
-    <t>gita.nasution55@outlook.com</t>
-  </si>
-  <si>
-    <t>irfan.santoso944@gmail.com</t>
-  </si>
-  <si>
-    <t>indah.saputra104@gmail.com</t>
-  </si>
-  <si>
-    <t>eko.kusuma887@outlook.com</t>
-  </si>
-  <si>
-    <t>eko.pane227@outlook.com</t>
-  </si>
-  <si>
-    <t>gilang.rahayu752@outlook.com</t>
-  </si>
-  <si>
-    <t>rina.nugroho236@gmail.com</t>
-  </si>
-  <si>
-    <t>citra.setiawan654@gmail.com</t>
-  </si>
-  <si>
-    <t>putri.firmansyah722@gmail.com</t>
-  </si>
-  <si>
-    <t>agus.nasution615@gmail.com</t>
-  </si>
-  <si>
-    <t>nur.santoso953@gmail.com</t>
-  </si>
-  <si>
-    <t>sari.lestari706@outlook.com</t>
-  </si>
-  <si>
-    <t>lestari.tanjung401@gmail.com</t>
-  </si>
-  <si>
-    <t>fitri.sitompul136@gmail.com</t>
-  </si>
-  <si>
-    <t>wahyu.purnomo929@gmail.com</t>
-  </si>
-  <si>
-    <t>oki.rahayu844@gmail.com</t>
-  </si>
-  <si>
-    <t>wulan.wijaya969@gmail.com</t>
-  </si>
-  <si>
-    <t>irfan.wijaya673@gmail.com</t>
-  </si>
-  <si>
-    <t>yoga.pane475@outlook.com</t>
-  </si>
-  <si>
-    <t>vina.purnomo192@outlook.com; indah.syahputra777@gmail.com</t>
-  </si>
-  <si>
-    <t>dewi.simanjuntak858@gmail.com</t>
-  </si>
-  <si>
-    <t>zaki.pane127@gmail.com</t>
-  </si>
-  <si>
-    <t>agus.halim86@yahoo.co.id</t>
-  </si>
-  <si>
-    <t>agus.nugroho89@yahoo.co.id</t>
-  </si>
-  <si>
-    <t>andi.purnomo234@gmail.com</t>
-  </si>
-  <si>
-    <t>joko.harahap511@gmail.com</t>
-  </si>
-  <si>
-    <t>nanda.marpaung438@gmail.com</t>
-  </si>
-  <si>
-    <t>irfan.tanjung184@gmail.com</t>
-  </si>
-  <si>
-    <t>fitri.utomo268@gmail.com</t>
-  </si>
-  <si>
-    <t>eko.nasution871@yahoo.co.id</t>
-  </si>
-  <si>
-    <t>maya.lestari694@gmail.com</t>
-  </si>
-  <si>
-    <t>eko.wibowo163@gmail.com</t>
-  </si>
-  <si>
-    <t>mega.rahayu969@gmail.com</t>
-  </si>
-  <si>
-    <t>dimas.pane811@gmail.com</t>
-  </si>
-  <si>
-    <t>nanda.pratama841@yahoo.co.id</t>
-  </si>
-  <si>
-    <t>dimas.siregar658@gmail.com</t>
-  </si>
-  <si>
-    <t>fajar.purnomo953@gmail.com</t>
-  </si>
-  <si>
-    <t>agus.hakim526@gmial.com</t>
-  </si>
-  <si>
-    <t>putri.lestari568@yahoo.co.id</t>
-  </si>
-  <si>
-    <t>joko.wibowo645@yahoo.co.id</t>
-  </si>
-  <si>
-    <t>dewi.purnomo638@gmail.com</t>
-  </si>
-  <si>
-    <t>sari.wijaya789@outlook.com</t>
-  </si>
-  <si>
-    <t>bayu.hakim696@gmail.com</t>
-  </si>
-  <si>
-    <t>nanda.ramadhan287@outlook.com</t>
-  </si>
-  <si>
-    <t>bayu.harahap869@yahoo.co.id</t>
-  </si>
-  <si>
-    <t>putri.sitompul57@gmail.com</t>
-  </si>
-  <si>
-    <t>irfan.gunawan138@gmail.com</t>
-  </si>
-  <si>
-    <t>wahyu.tanjung859@gmail.com</t>
-  </si>
-  <si>
-    <t>rizky.daeng504@yahoo.co.id</t>
-  </si>
-  <si>
-    <t>mega.wibowo950@yahoo.co.id</t>
-  </si>
-  <si>
-    <t>putri.rahayu941@gmail.com</t>
-  </si>
-  <si>
-    <t>fitri.nugroho227@gmail.com</t>
-  </si>
-  <si>
-    <t>joko.utomo267@outlook.com</t>
-  </si>
-  <si>
-    <t>joko.nasution268@yahoo.co.id</t>
-  </si>
-  <si>
-    <t>laras.wibowo869@gmail.com</t>
-  </si>
-  <si>
-    <t>surya.santoso798@gmail.com</t>
-  </si>
-  <si>
-    <t>eko.pratama215@gmail.com</t>
-  </si>
-  <si>
-    <t>lestari.pratama107@gmail.com</t>
-  </si>
-  <si>
-    <t>mega.pratama75@gmail.com</t>
-  </si>
-  <si>
-    <t>gita.harahap520@outlook.com</t>
-  </si>
-  <si>
-    <t>irfan.firmansyah131@yahoo.co.id</t>
-  </si>
-  <si>
-    <t>budi.wibowo941@gmail.com</t>
-  </si>
-  <si>
-    <t>putri.tanjung36@gmail.com</t>
-  </si>
-  <si>
-    <t>dimas.sitompul890@gmail.com</t>
-  </si>
-  <si>
-    <t>mega.nasution5@gmail.com</t>
-  </si>
-  <si>
-    <t>fitri.syahputra263@gmail.com</t>
-  </si>
-  <si>
-    <t>sari.nasution814@gmail.com</t>
-  </si>
-  <si>
-    <t>laras.simanjuntak14@outlook.com</t>
-  </si>
-  <si>
-    <t>surya.hidayat910@gmail.com</t>
-  </si>
-  <si>
-    <t>rahmat.firmansyah974@gmail.com</t>
-  </si>
-  <si>
-    <t>dimas.ramadhan647@gmail.com</t>
-  </si>
-  <si>
-    <t>gilang.rahayu567@outlook.com</t>
-  </si>
-  <si>
-    <t>laras.nasution838@gmail.com</t>
-  </si>
-  <si>
-    <t>rahmat.hakim508@yahoo.co.id</t>
-  </si>
-  <si>
-    <t>wahyu.marpaung230@outlook.com</t>
-  </si>
-  <si>
-    <t>gilang.purnomo421@gmail.com</t>
-  </si>
-  <si>
-    <t>dimas.susanto703@gmail.com</t>
-  </si>
-  <si>
-    <t>hana.nugroho214@outlook.com</t>
-  </si>
-  <si>
-    <t>lestari.tanjung978@outlook.com</t>
-  </si>
-  <si>
-    <t>joko.tanjung869@outlook.com</t>
-  </si>
-  <si>
-    <t>bayu.susanto849@yahoo.co.id</t>
-  </si>
-  <si>
-    <t>gilang.wijaya476@gmail.com</t>
-  </si>
-  <si>
-    <t>vina.setiawan486@yahoo.co.id</t>
-  </si>
-  <si>
-    <t>rina.utomo103@gmail.com</t>
-  </si>
-  <si>
-    <t>maya.permana531@gmail.com</t>
-  </si>
-  <si>
-    <t>utami.siregar3@gmail.com</t>
-  </si>
-  <si>
-    <t>lestari.daeng107@gmail.com</t>
-  </si>
-  <si>
-    <t>mega.utomo870@gmail.com</t>
-  </si>
-  <si>
-    <t>hana.utomo103@outlook.com</t>
-  </si>
-  <si>
-    <t>putri.purnomo589@yahoo.co.id</t>
-  </si>
-  <si>
-    <t>utami.wibowo65@yahoo.co.id</t>
+    <t>dimas.nasution608@outlook.example</t>
+  </si>
+  <si>
+    <t>vina.saputra573@gmail.example</t>
+  </si>
+  <si>
+    <t>tika.susanto926@gmail.example</t>
+  </si>
+  <si>
+    <t>nur.lestari650@gmail.example</t>
+  </si>
+  <si>
+    <t>joko.setiawan270@gmail.example</t>
+  </si>
+  <si>
+    <t>joko.nugroho688@gmail.example</t>
+  </si>
+  <si>
+    <t>rahmat.siregar337@gmail.example</t>
+  </si>
+  <si>
+    <t>budi.siregar667@gmail.example</t>
+  </si>
+  <si>
+    <t>yuni.ramadhan958@gmail.example</t>
+  </si>
+  <si>
+    <t>vina.setiawan655@outlook.example</t>
+  </si>
+  <si>
+    <t>budi.simanjuntak706@outlook.example</t>
+  </si>
+  <si>
+    <t>tika.firmansyah424@gmail.example</t>
+  </si>
+  <si>
+    <t>lestari.nugroho532@gmail.example</t>
+  </si>
+  <si>
+    <t>citra.siregar111@outlook.example</t>
+  </si>
+  <si>
+    <t>bayu.utomo296@gmail.example</t>
+  </si>
+  <si>
+    <t>vina.permana689@gmail.example</t>
+  </si>
+  <si>
+    <t>laras.firmansyah350@outlook.example</t>
+  </si>
+  <si>
+    <t>kartika.halim174@outlook.example</t>
+  </si>
+  <si>
+    <t>kartika.nugroho952@gmail.example</t>
+  </si>
+  <si>
+    <t>wahyu.gunawan107@outlook.example</t>
+  </si>
+  <si>
+    <t>irfan.sitompul545@yahoo.example</t>
+  </si>
+  <si>
+    <t>fitri.santoso810@outlook.example</t>
+  </si>
+  <si>
+    <t>surya.setiawan771@gmail.example</t>
+  </si>
+  <si>
+    <t>gilang.pratama510@outlook.example</t>
+  </si>
+  <si>
+    <t>surya.daeng364@outlook.example</t>
+  </si>
+  <si>
+    <t>andi.setiawan238.old@gmail.example</t>
+  </si>
+  <si>
+    <t>tika.marpaung805@outlook.example</t>
+  </si>
+  <si>
+    <t>mega.marpaung269@gmail.example</t>
+  </si>
+  <si>
+    <t>hendra.sitompul513@yahoo.example</t>
+  </si>
+  <si>
+    <t>mega.firmansyah422@gmail.example</t>
+  </si>
+  <si>
+    <t>rizky.firmansyah364@gmail.example</t>
+  </si>
+  <si>
+    <t>joko.wijaya663@gmail.example</t>
+  </si>
+  <si>
+    <t>fitri.rahayu13@outlook.example</t>
+  </si>
+  <si>
+    <t>yoga.lestari340@yahoo.example</t>
+  </si>
+  <si>
+    <t>yuni.saputra879@yahoo.example</t>
+  </si>
+  <si>
+    <t>oki.hakim372@outlook.example</t>
+  </si>
+  <si>
+    <t>zaki.nasution210@yahoo.example</t>
+  </si>
+  <si>
+    <t>rahmat.siregar757@gmail.example</t>
+  </si>
+  <si>
+    <t>gita.hidayat136@gmail.example</t>
+  </si>
+  <si>
+    <t>laras.ramadhan779@yahoo.example</t>
+  </si>
+  <si>
+    <t>tika.wijaya764@gmail.example</t>
+  </si>
+  <si>
+    <t>vina.harahap695@gmail.example</t>
+  </si>
+  <si>
+    <t>lestari.lestari789@gmail.example</t>
+  </si>
+  <si>
+    <t>gilang.daeng87@gmail.example</t>
+  </si>
+  <si>
+    <t>mega.syahputra515@gmail.example</t>
+  </si>
+  <si>
+    <t>irfan.lestari524@gmail.example</t>
+  </si>
+  <si>
+    <t>rina.hakim486@gmail.example</t>
+  </si>
+  <si>
+    <t>utami.saputra534@gmail.example</t>
+  </si>
+  <si>
+    <t>eko.firmansyah611@gmail.example</t>
+  </si>
+  <si>
+    <t>gilang.halim260@gmail.example</t>
+  </si>
+  <si>
+    <t>yuni.daeng514@yahoo.example</t>
+  </si>
+  <si>
+    <t>eko.simanjuntak230@outlook.example</t>
+  </si>
+  <si>
+    <t>taufik.purnomo473@gmail.example</t>
+  </si>
+  <si>
+    <t>nur.kusuma124@gmail.example</t>
+  </si>
+  <si>
+    <t>bayu.setiawan607@gmail.example</t>
+  </si>
+  <si>
+    <t>bayu.gunawan728@outlook.example</t>
+  </si>
+  <si>
+    <t>zaki.purnomo501@gmail.example</t>
+  </si>
+  <si>
+    <t>eko.nasution202@gmail.example</t>
+  </si>
+  <si>
+    <t>dewi.hidayat608@gmail.example</t>
+  </si>
+  <si>
+    <t>gita.nasution55@outlook.example</t>
+  </si>
+  <si>
+    <t>irfan.santoso944@gmail.example</t>
+  </si>
+  <si>
+    <t>indah.saputra104@gmail.example</t>
+  </si>
+  <si>
+    <t>eko.kusuma887@outlook.example</t>
+  </si>
+  <si>
+    <t>eko.pane227@outlook.example</t>
+  </si>
+  <si>
+    <t>gilang.rahayu752@outlook.example</t>
+  </si>
+  <si>
+    <t>rina.nugroho236@gmail.example</t>
+  </si>
+  <si>
+    <t>citra.setiawan654@gmail.example</t>
+  </si>
+  <si>
+    <t>putri.firmansyah722@gmail.example</t>
+  </si>
+  <si>
+    <t>agus.nasution615@gmail.example</t>
+  </si>
+  <si>
+    <t>nur.santoso953@gmail.example</t>
+  </si>
+  <si>
+    <t>sari.lestari706@outlook.example</t>
+  </si>
+  <si>
+    <t>lestari.tanjung401@gmail.example</t>
+  </si>
+  <si>
+    <t>fitri.sitompul136@gmail.example</t>
+  </si>
+  <si>
+    <t>wahyu.purnomo929@gmail.example</t>
+  </si>
+  <si>
+    <t>oki.rahayu844@gmail.example</t>
+  </si>
+  <si>
+    <t>wulan.wijaya969@gmail.example</t>
+  </si>
+  <si>
+    <t>irfan.wijaya673@gmail.example</t>
+  </si>
+  <si>
+    <t>yoga.pane475@outlook.example</t>
+  </si>
+  <si>
+    <t>vina.purnomo192@outlook.example; indah.syahputra777@gmail.example</t>
+  </si>
+  <si>
+    <t>dewi.simanjuntak858@gmail.example</t>
+  </si>
+  <si>
+    <t>zaki.pane127@gmail.example</t>
+  </si>
+  <si>
+    <t>agus.halim86@yahoo.example</t>
+  </si>
+  <si>
+    <t>agus.nugroho89@yahoo.example</t>
+  </si>
+  <si>
+    <t>andi.purnomo234@gmail.example</t>
+  </si>
+  <si>
+    <t>joko.harahap511@gmail.example</t>
+  </si>
+  <si>
+    <t>nanda.marpaung438@gmail.example</t>
+  </si>
+  <si>
+    <t>irfan.tanjung184@gmail.example</t>
+  </si>
+  <si>
+    <t>fitri.utomo268@gmail.example</t>
+  </si>
+  <si>
+    <t>eko.nasution871@yahoo.example</t>
+  </si>
+  <si>
+    <t>maya.lestari694@gmail.example</t>
+  </si>
+  <si>
+    <t>eko.wibowo163@gmail.example</t>
+  </si>
+  <si>
+    <t>mega.rahayu969@gmail.example</t>
+  </si>
+  <si>
+    <t>dimas.pane811@gmail.example</t>
+  </si>
+  <si>
+    <t>nanda.pratama841@yahoo.example</t>
+  </si>
+  <si>
+    <t>dimas.siregar658@gmail.example</t>
+  </si>
+  <si>
+    <t>fajar.purnomo953@gmail.example</t>
+  </si>
+  <si>
+    <t>agus.hakim526@gmial.example</t>
+  </si>
+  <si>
+    <t>putri.lestari568@yahoo.example</t>
+  </si>
+  <si>
+    <t>joko.wibowo645@yahoo.example</t>
+  </si>
+  <si>
+    <t>dewi.purnomo638@gmail.example</t>
+  </si>
+  <si>
+    <t>sari.wijaya789@outlook.example</t>
+  </si>
+  <si>
+    <t>bayu.hakim696@gmail.example</t>
+  </si>
+  <si>
+    <t>nanda.ramadhan287@outlook.example</t>
+  </si>
+  <si>
+    <t>bayu.harahap869@yahoo.example</t>
+  </si>
+  <si>
+    <t>putri.sitompul57@gmail.example</t>
+  </si>
+  <si>
+    <t>irfan.gunawan138@gmail.example</t>
+  </si>
+  <si>
+    <t>wahyu.tanjung859@gmail.example</t>
+  </si>
+  <si>
+    <t>rizky.daeng504@yahoo.example</t>
+  </si>
+  <si>
+    <t>mega.wibowo950@yahoo.example</t>
+  </si>
+  <si>
+    <t>putri.rahayu941@gmail.example</t>
+  </si>
+  <si>
+    <t>fitri.nugroho227@gmail.example</t>
+  </si>
+  <si>
+    <t>joko.utomo267@outlook.example</t>
+  </si>
+  <si>
+    <t>joko.nasution268@yahoo.example</t>
+  </si>
+  <si>
+    <t>laras.wibowo869@gmail.example</t>
+  </si>
+  <si>
+    <t>surya.santoso798@gmail.example</t>
+  </si>
+  <si>
+    <t>eko.pratama215@gmail.example</t>
+  </si>
+  <si>
+    <t>lestari.pratama107@gmail.example</t>
+  </si>
+  <si>
+    <t>mega.pratama75@gmail.example</t>
+  </si>
+  <si>
+    <t>gita.harahap520@outlook.example</t>
+  </si>
+  <si>
+    <t>irfan.firmansyah131@yahoo.example</t>
+  </si>
+  <si>
+    <t>budi.wibowo941@gmail.example</t>
+  </si>
+  <si>
+    <t>putri.tanjung36@gmail.example</t>
+  </si>
+  <si>
+    <t>dimas.sitompul890@gmail.example</t>
+  </si>
+  <si>
+    <t>mega.nasution5@gmail.example</t>
+  </si>
+  <si>
+    <t>fitri.syahputra263@gmail.example</t>
+  </si>
+  <si>
+    <t>sari.nasution814@gmail.example</t>
+  </si>
+  <si>
+    <t>laras.simanjuntak14@outlook.example</t>
+  </si>
+  <si>
+    <t>surya.hidayat910@gmail.example</t>
+  </si>
+  <si>
+    <t>rahmat.firmansyah974@gmail.example</t>
+  </si>
+  <si>
+    <t>dimas.ramadhan647@gmail.example</t>
+  </si>
+  <si>
+    <t>gilang.rahayu567@outlook.example</t>
+  </si>
+  <si>
+    <t>laras.nasution838@gmail.example</t>
+  </si>
+  <si>
+    <t>rahmat.hakim508@yahoo.example</t>
+  </si>
+  <si>
+    <t>wahyu.marpaung230@outlook.example</t>
+  </si>
+  <si>
+    <t>gilang.purnomo421@gmail.example</t>
+  </si>
+  <si>
+    <t>dimas.susanto703@gmail.example</t>
+  </si>
+  <si>
+    <t>hana.nugroho214@outlook.example</t>
+  </si>
+  <si>
+    <t>lestari.tanjung978@outlook.example</t>
+  </si>
+  <si>
+    <t>joko.tanjung869@outlook.example</t>
+  </si>
+  <si>
+    <t>bayu.susanto849@yahoo.example</t>
+  </si>
+  <si>
+    <t>gilang.wijaya476@gmail.example</t>
+  </si>
+  <si>
+    <t>vina.setiawan486@yahoo.example</t>
+  </si>
+  <si>
+    <t>rina.utomo103@gmail.example</t>
+  </si>
+  <si>
+    <t>maya.permana531@gmail.example</t>
+  </si>
+  <si>
+    <t>utami.siregar3@gmail.example</t>
+  </si>
+  <si>
+    <t>lestari.daeng107@gmail.example</t>
+  </si>
+  <si>
+    <t>mega.utomo870@gmail.example</t>
+  </si>
+  <si>
+    <t>hana.utomo103@outlook.example</t>
+  </si>
+  <si>
+    <t>putri.purnomo589@yahoo.example</t>
+  </si>
+  <si>
+    <t>utami.wibowo65@yahoo.example</t>
   </si>
   <si>
     <t>BDG</t>
@@ -1402,7 +1402,7 @@
     <t>MATURITY</t>
   </si>
   <si>
-    <t>mks.staff@gmail.com</t>
+    <t>mks.staff@gmail.example</t>
   </si>
 </sst>
 </file>

</xml_diff>